<commit_message>
derbies back to 2022
</commit_message>
<xml_diff>
--- a/data/sources/derbies.xlsx
+++ b/data/sources/derbies.xlsx
@@ -8,25 +8,36 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofwa-my.sharepoint.com/personal/tyler_garber_dfw_wa_gov/Documents/sport_harvest/sport/sport_harvest_estimator/data/sources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="42" documentId="11_F25DC773A252ABDACC1048A0A95D59F65BDE58F6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{68D376A2-0C67-4E95-9265-B466E8478F37}"/>
+  <xr:revisionPtr revIDLastSave="125" documentId="11_F25DC773A252ABDACC1048A0A95D59F65BDE58F6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4AEE74E1-424B-4E3A-870E-E7C3E2F160E8}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-105" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
     <sheet name="readme" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="20">
   <si>
     <t>Derbies don't get captured in the in-season estimates. For a full accounting take them from the in-season season sheet and paste in the `data` tab.</t>
   </si>
@@ -65,19 +76,45 @@
   </si>
   <si>
     <t>coho_104_uk_ret</t>
+  </si>
+  <si>
+    <t>RCAW Derby</t>
+  </si>
+  <si>
+    <t>Gig Harbor Salmon Derby</t>
+  </si>
+  <si>
+    <t>Whidbey Isl Coho Derby</t>
+  </si>
+  <si>
+    <t>Kiwanis Kingston Coho Derby</t>
+  </si>
+  <si>
+    <t>Reserection Coho Derby</t>
+  </si>
+  <si>
+    <t>S. King Co PSA Derby</t>
+  </si>
+  <si>
+    <t>Gig Harbor PSA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -97,18 +134,21 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 6" xfId="1" xr:uid="{A9DB1EA0-4EEC-451F-B957-4826AE7AA2BC}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -386,7 +426,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="4" width="9.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -642,6 +682,719 @@
         <v>5</v>
       </c>
       <c r="G11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>82</v>
+      </c>
+      <c r="B12" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="1">
+        <v>45542</v>
+      </c>
+      <c r="D12" s="1">
+        <v>45542</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>10</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>82</v>
+      </c>
+      <c r="B13" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" s="1">
+        <v>45556</v>
+      </c>
+      <c r="D13" s="1">
+        <v>45557</v>
+      </c>
+      <c r="E13">
+        <v>96</v>
+      </c>
+      <c r="F13">
+        <v>31</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>81</v>
+      </c>
+      <c r="B14" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="1">
+        <v>45542</v>
+      </c>
+      <c r="D14" s="1">
+        <v>45542</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>81</v>
+      </c>
+      <c r="B15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="1">
+        <v>45556</v>
+      </c>
+      <c r="D15" s="1">
+        <v>45557</v>
+      </c>
+      <c r="E15">
+        <v>2</v>
+      </c>
+      <c r="F15">
+        <v>16</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>11</v>
+      </c>
+      <c r="B16" t="s">
+        <v>13</v>
+      </c>
+      <c r="C16" s="1">
+        <v>45499</v>
+      </c>
+      <c r="D16" s="1">
+        <v>45499</v>
+      </c>
+      <c r="E16">
+        <v>2</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="G16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>11</v>
+      </c>
+      <c r="B17" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" s="1">
+        <v>45507</v>
+      </c>
+      <c r="D17" s="1">
+        <v>45507</v>
+      </c>
+      <c r="E17">
+        <v>0</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+      <c r="G17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>10</v>
+      </c>
+      <c r="B18" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" s="1">
+        <v>45499</v>
+      </c>
+      <c r="D18" s="1">
+        <v>45499</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>10</v>
+      </c>
+      <c r="B19" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" s="1">
+        <v>45542</v>
+      </c>
+      <c r="D19" s="1">
+        <v>45542</v>
+      </c>
+      <c r="E19">
+        <v>142</v>
+      </c>
+      <c r="F19">
+        <v>176</v>
+      </c>
+      <c r="G19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>10</v>
+      </c>
+      <c r="B20" t="s">
+        <v>15</v>
+      </c>
+      <c r="C20" s="1">
+        <v>45548</v>
+      </c>
+      <c r="D20" s="1">
+        <v>45550</v>
+      </c>
+      <c r="E20">
+        <v>40</v>
+      </c>
+      <c r="F20">
+        <v>42</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>10</v>
+      </c>
+      <c r="B21" t="s">
+        <v>16</v>
+      </c>
+      <c r="C21" s="1">
+        <v>45556</v>
+      </c>
+      <c r="D21" s="1">
+        <v>45556</v>
+      </c>
+      <c r="E21">
+        <v>51</v>
+      </c>
+      <c r="F21">
+        <v>120</v>
+      </c>
+      <c r="G21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>10</v>
+      </c>
+      <c r="B22" t="s">
+        <v>8</v>
+      </c>
+      <c r="C22" s="1">
+        <v>45556</v>
+      </c>
+      <c r="D22" s="1">
+        <v>45557</v>
+      </c>
+      <c r="E22">
+        <v>139</v>
+      </c>
+      <c r="F22">
+        <v>271</v>
+      </c>
+      <c r="G22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>9</v>
+      </c>
+      <c r="B23" t="s">
+        <v>7</v>
+      </c>
+      <c r="C23" s="1">
+        <v>45542</v>
+      </c>
+      <c r="D23" s="1">
+        <v>45542</v>
+      </c>
+      <c r="E23">
+        <v>93</v>
+      </c>
+      <c r="F23">
+        <v>2</v>
+      </c>
+      <c r="G23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>9</v>
+      </c>
+      <c r="B24" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" s="1">
+        <v>45556</v>
+      </c>
+      <c r="D24" s="1">
+        <v>45556</v>
+      </c>
+      <c r="E24">
+        <v>24</v>
+      </c>
+      <c r="F24">
+        <v>9</v>
+      </c>
+      <c r="G24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>9</v>
+      </c>
+      <c r="B25" t="s">
+        <v>8</v>
+      </c>
+      <c r="C25" s="1">
+        <v>45556</v>
+      </c>
+      <c r="D25" s="1">
+        <v>45557</v>
+      </c>
+      <c r="E25">
+        <v>137</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+      <c r="G25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>11</v>
+      </c>
+      <c r="B26" t="s">
+        <v>13</v>
+      </c>
+      <c r="C26" s="1">
+        <v>45870</v>
+      </c>
+      <c r="D26" s="1">
+        <v>45870</v>
+      </c>
+      <c r="E26" s="2">
+        <v>1.0275229357798166</v>
+      </c>
+      <c r="F26" s="2">
+        <v>0.51376146788990829</v>
+      </c>
+      <c r="G26" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>11</v>
+      </c>
+      <c r="B27" t="s">
+        <v>14</v>
+      </c>
+      <c r="C27" s="1">
+        <v>45507</v>
+      </c>
+      <c r="D27" s="1">
+        <v>45507</v>
+      </c>
+      <c r="E27" s="2">
+        <v>3.52112676056338</v>
+      </c>
+      <c r="F27" s="2">
+        <v>1.4084507042253522</v>
+      </c>
+      <c r="G27" s="2">
+        <v>0.35211267605633806</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>10</v>
+      </c>
+      <c r="B28" t="s">
+        <v>13</v>
+      </c>
+      <c r="C28" s="1">
+        <v>45870</v>
+      </c>
+      <c r="D28" s="1">
+        <v>45870</v>
+      </c>
+      <c r="E28">
+        <v>0</v>
+      </c>
+      <c r="F28">
+        <v>0</v>
+      </c>
+      <c r="G28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>10</v>
+      </c>
+      <c r="B29" t="s">
+        <v>7</v>
+      </c>
+      <c r="C29" s="1">
+        <v>45906</v>
+      </c>
+      <c r="D29" s="1">
+        <v>45906</v>
+      </c>
+      <c r="E29">
+        <v>52</v>
+      </c>
+      <c r="F29">
+        <v>66</v>
+      </c>
+      <c r="G29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>10</v>
+      </c>
+      <c r="B30" t="s">
+        <v>16</v>
+      </c>
+      <c r="C30" s="1">
+        <v>45920</v>
+      </c>
+      <c r="D30" s="1">
+        <v>45920</v>
+      </c>
+      <c r="E30">
+        <v>6</v>
+      </c>
+      <c r="F30">
+        <v>3</v>
+      </c>
+      <c r="G30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>10</v>
+      </c>
+      <c r="B31" t="s">
+        <v>8</v>
+      </c>
+      <c r="C31" s="1">
+        <v>45920</v>
+      </c>
+      <c r="D31" s="1">
+        <v>45921</v>
+      </c>
+      <c r="E31">
+        <v>153</v>
+      </c>
+      <c r="F31">
+        <v>140</v>
+      </c>
+      <c r="G31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>9</v>
+      </c>
+      <c r="B32" t="s">
+        <v>16</v>
+      </c>
+      <c r="C32" s="1">
+        <v>45185</v>
+      </c>
+      <c r="D32" s="1">
+        <v>45185</v>
+      </c>
+      <c r="E32">
+        <v>26</v>
+      </c>
+      <c r="F32">
+        <v>0</v>
+      </c>
+      <c r="G32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>9</v>
+      </c>
+      <c r="B33" t="s">
+        <v>8</v>
+      </c>
+      <c r="C33" s="1">
+        <v>45192</v>
+      </c>
+      <c r="D33" s="1">
+        <v>45192</v>
+      </c>
+      <c r="E33">
+        <v>257</v>
+      </c>
+      <c r="F33">
+        <v>419</v>
+      </c>
+      <c r="G33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>10</v>
+      </c>
+      <c r="B34" t="s">
+        <v>16</v>
+      </c>
+      <c r="C34" s="1">
+        <v>45185</v>
+      </c>
+      <c r="D34" s="1">
+        <v>45185</v>
+      </c>
+      <c r="E34">
+        <v>29</v>
+      </c>
+      <c r="F34">
+        <v>32</v>
+      </c>
+      <c r="G34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>10</v>
+      </c>
+      <c r="B35" t="s">
+        <v>8</v>
+      </c>
+      <c r="C35" s="1">
+        <v>45192</v>
+      </c>
+      <c r="D35" s="1">
+        <v>45192</v>
+      </c>
+      <c r="E35">
+        <v>13</v>
+      </c>
+      <c r="F35">
+        <v>8</v>
+      </c>
+      <c r="G35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>82</v>
+      </c>
+      <c r="B36" t="s">
+        <v>8</v>
+      </c>
+      <c r="C36" s="1">
+        <v>45192</v>
+      </c>
+      <c r="D36" s="1">
+        <v>45192</v>
+      </c>
+      <c r="E36">
+        <v>68</v>
+      </c>
+      <c r="F36">
+        <v>95</v>
+      </c>
+      <c r="G36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>7</v>
+      </c>
+      <c r="B37" t="s">
+        <v>17</v>
+      </c>
+      <c r="C37" s="1">
+        <v>44792</v>
+      </c>
+      <c r="D37" s="1">
+        <v>44793</v>
+      </c>
+      <c r="E37">
+        <v>7</v>
+      </c>
+      <c r="F37">
+        <v>0</v>
+      </c>
+      <c r="G37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>9</v>
+      </c>
+      <c r="B38" t="s">
+        <v>8</v>
+      </c>
+      <c r="C38" s="1">
+        <v>44828</v>
+      </c>
+      <c r="D38" s="1">
+        <v>44829</v>
+      </c>
+      <c r="E38">
+        <v>322</v>
+      </c>
+      <c r="F38">
+        <v>0</v>
+      </c>
+      <c r="G38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>10</v>
+      </c>
+      <c r="B39" t="s">
+        <v>8</v>
+      </c>
+      <c r="C39" s="1">
+        <v>44828</v>
+      </c>
+      <c r="D39" s="1">
+        <v>44829</v>
+      </c>
+      <c r="E39">
+        <v>638</v>
+      </c>
+      <c r="F39">
+        <v>0</v>
+      </c>
+      <c r="G39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>11</v>
+      </c>
+      <c r="B40" t="s">
+        <v>13</v>
+      </c>
+      <c r="C40" s="1">
+        <v>44776</v>
+      </c>
+      <c r="D40" s="1">
+        <v>44776</v>
+      </c>
+      <c r="E40">
+        <v>0</v>
+      </c>
+      <c r="F40">
+        <v>0</v>
+      </c>
+      <c r="G40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>11</v>
+      </c>
+      <c r="B41" t="s">
+        <v>18</v>
+      </c>
+      <c r="C41" s="1">
+        <v>44779</v>
+      </c>
+      <c r="D41" s="1">
+        <v>44779</v>
+      </c>
+      <c r="E41">
+        <v>15</v>
+      </c>
+      <c r="F41">
+        <v>0</v>
+      </c>
+      <c r="G41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>11</v>
+      </c>
+      <c r="B42" t="s">
+        <v>19</v>
+      </c>
+      <c r="C42" s="1">
+        <v>44786</v>
+      </c>
+      <c r="D42" s="1">
+        <v>44786</v>
+      </c>
+      <c r="E42">
+        <v>15</v>
+      </c>
+      <c r="F42">
+        <v>0</v>
+      </c>
+      <c r="G42">
         <v>0</v>
       </c>
     </row>
@@ -656,55 +1409,55 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
+      <c r="A6" s="3"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>